<commit_message>
Decision for GLYCO-2025-00103.R1 feedback edits
</commit_message>
<xml_diff>
--- a/dataloader/data/GlycoEnzOntoDB.xlsx
+++ b/dataloader/data/GlycoEnzOntoDB.xlsx
@@ -2034,7 +2034,7 @@
     <t>Glycosylation Regulation</t>
   </si>
   <si>
-    <t>2</t>
+    <t>EC 2.-</t>
   </si>
   <si>
     <t>2.4</t>
@@ -2055,7 +2055,7 @@
     <t>2.4.1.37</t>
   </si>
   <si>
-    <t>3</t>
+    <t>EC 3.-</t>
   </si>
   <si>
     <t>3.5</t>
@@ -2241,7 +2241,7 @@
     <t>2.4.1.174</t>
   </si>
   <si>
-    <t>1</t>
+    <t>EC 1.-</t>
   </si>
   <si>
     <t>1.8</t>
@@ -2259,7 +2259,7 @@
     <t>2.4.1.83</t>
   </si>
   <si>
-    <t>5</t>
+    <t>EC 5.-</t>
   </si>
   <si>
     <t>5.1</t>
@@ -2397,7 +2397,7 @@
     <t>5.1.3.17</t>
   </si>
   <si>
-    <t>4</t>
+    <t>EC 4.-</t>
   </si>
   <si>
     <t>4.2</t>
@@ -2763,7 +2763,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -2771,6 +2771,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -20517,7 +20520,7 @@
       </c>
     </row>
     <row r="990" ht="15.75" customHeight="1">
-      <c r="L990" s="2" t="s">
+      <c r="L990" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M990" s="2" t="s">
@@ -20534,7 +20537,7 @@
       </c>
     </row>
     <row r="991" ht="15.75" customHeight="1">
-      <c r="L991" s="2" t="s">
+      <c r="L991" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M991" s="2" t="s">
@@ -20551,7 +20554,7 @@
       </c>
     </row>
     <row r="992" ht="15.75" customHeight="1">
-      <c r="L992" s="2" t="s">
+      <c r="L992" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M992" s="2" t="s">
@@ -20566,7 +20569,7 @@
       </c>
     </row>
     <row r="993" ht="15.75" customHeight="1">
-      <c r="L993" s="2" t="s">
+      <c r="L993" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M993" s="2" t="s">
@@ -20583,7 +20586,7 @@
       </c>
     </row>
     <row r="994" ht="15.75" customHeight="1">
-      <c r="L994" s="2" t="s">
+      <c r="L994" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M994" s="2" t="s">
@@ -20600,7 +20603,7 @@
       </c>
     </row>
     <row r="995" ht="15.75" customHeight="1">
-      <c r="L995" s="2" t="s">
+      <c r="L995" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M995" s="2" t="s">
@@ -20617,7 +20620,7 @@
       </c>
     </row>
     <row r="996" ht="15.75" customHeight="1">
-      <c r="L996" s="2" t="s">
+      <c r="L996" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M996" s="2" t="s">
@@ -20634,7 +20637,7 @@
       </c>
     </row>
     <row r="997" ht="15.75" customHeight="1">
-      <c r="L997" s="2" t="s">
+      <c r="L997" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M997" s="2" t="s">
@@ -20651,7 +20654,7 @@
       </c>
     </row>
     <row r="998" ht="15.75" customHeight="1">
-      <c r="L998" s="2" t="s">
+      <c r="L998" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M998" s="2" t="s">
@@ -20668,7 +20671,7 @@
       </c>
     </row>
     <row r="999" ht="15.75" customHeight="1">
-      <c r="L999" s="2" t="s">
+      <c r="L999" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M999" s="2" t="s">
@@ -20685,7 +20688,7 @@
       </c>
     </row>
     <row r="1000" ht="15.75" customHeight="1">
-      <c r="L1000" s="2" t="s">
+      <c r="L1000" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1000" s="2" t="s">
@@ -20702,7 +20705,7 @@
       </c>
     </row>
     <row r="1001" ht="15.75" customHeight="1">
-      <c r="L1001" s="2" t="s">
+      <c r="L1001" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1001" s="2" t="s">
@@ -20719,7 +20722,7 @@
       </c>
     </row>
     <row r="1002" ht="15.75" customHeight="1">
-      <c r="L1002" s="2" t="s">
+      <c r="L1002" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1002" s="2" t="s">
@@ -20734,7 +20737,7 @@
       </c>
     </row>
     <row r="1003" ht="15.75" customHeight="1">
-      <c r="L1003" s="2" t="s">
+      <c r="L1003" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1003" s="2" t="s">
@@ -20751,7 +20754,7 @@
       </c>
     </row>
     <row r="1004" ht="15.75" customHeight="1">
-      <c r="L1004" s="2" t="s">
+      <c r="L1004" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1004" s="2" t="s">
@@ -20768,7 +20771,7 @@
       </c>
     </row>
     <row r="1005" ht="15.75" customHeight="1">
-      <c r="L1005" s="2" t="s">
+      <c r="L1005" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1005" s="2" t="s">
@@ -20785,7 +20788,7 @@
       </c>
     </row>
     <row r="1006" ht="15.75" customHeight="1">
-      <c r="L1006" s="2" t="s">
+      <c r="L1006" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1006" s="2" t="s">
@@ -20802,7 +20805,7 @@
       </c>
     </row>
     <row r="1007" ht="15.75" customHeight="1">
-      <c r="L1007" s="2" t="s">
+      <c r="L1007" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1007" s="2" t="s">
@@ -20819,7 +20822,7 @@
       </c>
     </row>
     <row r="1008" ht="15.75" customHeight="1">
-      <c r="L1008" s="2" t="s">
+      <c r="L1008" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1008" s="2" t="s">
@@ -20836,7 +20839,7 @@
       </c>
     </row>
     <row r="1009" ht="15.75" customHeight="1">
-      <c r="L1009" s="2" t="s">
+      <c r="L1009" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1009" s="2" t="s">
@@ -20853,7 +20856,7 @@
       </c>
     </row>
     <row r="1010" ht="15.75" customHeight="1">
-      <c r="L1010" s="2" t="s">
+      <c r="L1010" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1010" s="2" t="s">
@@ -20870,7 +20873,7 @@
       </c>
     </row>
     <row r="1011" ht="15.75" customHeight="1">
-      <c r="L1011" s="2" t="s">
+      <c r="L1011" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1011" s="2" t="s">
@@ -20887,7 +20890,7 @@
       </c>
     </row>
     <row r="1012" ht="15.75" customHeight="1">
-      <c r="L1012" s="2" t="s">
+      <c r="L1012" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1012" s="2" t="s">
@@ -20904,7 +20907,7 @@
       </c>
     </row>
     <row r="1013" ht="15.75" customHeight="1">
-      <c r="L1013" s="2" t="s">
+      <c r="L1013" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1013" s="2" t="s">
@@ -20921,7 +20924,7 @@
       </c>
     </row>
     <row r="1014" ht="15.75" customHeight="1">
-      <c r="L1014" s="2" t="s">
+      <c r="L1014" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1014" s="2" t="s">
@@ -20938,7 +20941,7 @@
       </c>
     </row>
     <row r="1015" ht="15.75" customHeight="1">
-      <c r="L1015" s="2" t="s">
+      <c r="L1015" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1015" s="2" t="s">
@@ -20955,7 +20958,7 @@
       </c>
     </row>
     <row r="1016" ht="15.75" customHeight="1">
-      <c r="L1016" s="2" t="s">
+      <c r="L1016" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1016" s="2" t="s">
@@ -20972,7 +20975,7 @@
       </c>
     </row>
     <row r="1017" ht="15.75" customHeight="1">
-      <c r="L1017" s="2" t="s">
+      <c r="L1017" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1017" s="2" t="s">
@@ -20989,7 +20992,7 @@
       </c>
     </row>
     <row r="1018" ht="15.75" customHeight="1">
-      <c r="L1018" s="2" t="s">
+      <c r="L1018" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1018" s="2" t="s">
@@ -21006,7 +21009,7 @@
       </c>
     </row>
     <row r="1019" ht="15.75" customHeight="1">
-      <c r="L1019" s="2" t="s">
+      <c r="L1019" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1019" s="2" t="s">
@@ -21023,7 +21026,7 @@
       </c>
     </row>
     <row r="1020" ht="15.75" customHeight="1">
-      <c r="L1020" s="2" t="s">
+      <c r="L1020" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1020" s="2" t="s">
@@ -21038,7 +21041,7 @@
       </c>
     </row>
     <row r="1021" ht="15.75" customHeight="1">
-      <c r="L1021" s="2" t="s">
+      <c r="L1021" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1021" s="2" t="s">
@@ -21055,7 +21058,7 @@
       </c>
     </row>
     <row r="1022" ht="15.75" customHeight="1">
-      <c r="L1022" s="2" t="s">
+      <c r="L1022" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1022" s="2" t="s">
@@ -21072,7 +21075,7 @@
       </c>
     </row>
     <row r="1023" ht="15.75" customHeight="1">
-      <c r="L1023" s="2" t="s">
+      <c r="L1023" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1023" s="2" t="s">
@@ -21089,7 +21092,7 @@
       </c>
     </row>
     <row r="1024" ht="15.75" customHeight="1">
-      <c r="L1024" s="2" t="s">
+      <c r="L1024" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1024" s="2" t="s">
@@ -21106,7 +21109,7 @@
       </c>
     </row>
     <row r="1025" ht="15.75" customHeight="1">
-      <c r="L1025" s="2" t="s">
+      <c r="L1025" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1025" s="2" t="s">
@@ -21121,7 +21124,7 @@
       </c>
     </row>
     <row r="1026" ht="15.75" customHeight="1">
-      <c r="L1026" s="2" t="s">
+      <c r="L1026" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1026" s="2" t="s">
@@ -21138,7 +21141,7 @@
       </c>
     </row>
     <row r="1027" ht="15.75" customHeight="1">
-      <c r="L1027" s="2" t="s">
+      <c r="L1027" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1027" s="2" t="s">
@@ -21155,7 +21158,7 @@
       </c>
     </row>
     <row r="1028" ht="15.75" customHeight="1">
-      <c r="L1028" s="2" t="s">
+      <c r="L1028" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1028" s="2" t="s">
@@ -21172,7 +21175,7 @@
       </c>
     </row>
     <row r="1029" ht="15.75" customHeight="1">
-      <c r="L1029" s="2" t="s">
+      <c r="L1029" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1029" s="2" t="s">
@@ -21189,7 +21192,7 @@
       </c>
     </row>
     <row r="1030" ht="15.75" customHeight="1">
-      <c r="L1030" s="2" t="s">
+      <c r="L1030" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1030" s="2" t="s">
@@ -21206,7 +21209,7 @@
       </c>
     </row>
     <row r="1031" ht="15.75" customHeight="1">
-      <c r="L1031" s="2" t="s">
+      <c r="L1031" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1031" s="2" t="s">
@@ -21223,7 +21226,7 @@
       </c>
     </row>
     <row r="1032" ht="15.75" customHeight="1">
-      <c r="L1032" s="2" t="s">
+      <c r="L1032" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1032" s="2" t="s">
@@ -21238,7 +21241,7 @@
       </c>
     </row>
     <row r="1033" ht="15.75" customHeight="1">
-      <c r="L1033" s="2" t="s">
+      <c r="L1033" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1033" s="2" t="s">
@@ -21253,7 +21256,7 @@
       </c>
     </row>
     <row r="1034" ht="15.75" customHeight="1">
-      <c r="L1034" s="2" t="s">
+      <c r="L1034" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1034" s="2" t="s">
@@ -21270,7 +21273,7 @@
       </c>
     </row>
     <row r="1035" ht="15.75" customHeight="1">
-      <c r="L1035" s="2" t="s">
+      <c r="L1035" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1035" s="2" t="s">
@@ -21285,7 +21288,7 @@
       </c>
     </row>
     <row r="1036" ht="15.75" customHeight="1">
-      <c r="L1036" s="2" t="s">
+      <c r="L1036" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1036" s="2" t="s">
@@ -21302,7 +21305,7 @@
       </c>
     </row>
     <row r="1037" ht="15.75" customHeight="1">
-      <c r="L1037" s="2" t="s">
+      <c r="L1037" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1037" s="2" t="s">
@@ -21319,7 +21322,7 @@
       </c>
     </row>
     <row r="1038" ht="15.75" customHeight="1">
-      <c r="L1038" s="2" t="s">
+      <c r="L1038" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1038" s="2" t="s">
@@ -21336,7 +21339,7 @@
       </c>
     </row>
     <row r="1039" ht="15.75" customHeight="1">
-      <c r="L1039" s="2" t="s">
+      <c r="L1039" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1039" s="2" t="s">
@@ -21353,7 +21356,7 @@
       </c>
     </row>
     <row r="1040" ht="15.75" customHeight="1">
-      <c r="L1040" s="2" t="s">
+      <c r="L1040" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1040" s="2" t="s">
@@ -21370,7 +21373,7 @@
       </c>
     </row>
     <row r="1041" ht="15.75" customHeight="1">
-      <c r="L1041" s="2" t="s">
+      <c r="L1041" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1041" s="2" t="s">
@@ -21385,7 +21388,7 @@
       </c>
     </row>
     <row r="1042" ht="15.75" customHeight="1">
-      <c r="L1042" s="2" t="s">
+      <c r="L1042" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1042" s="2" t="s">
@@ -21402,7 +21405,7 @@
       </c>
     </row>
     <row r="1043" ht="15.75" customHeight="1">
-      <c r="L1043" s="2" t="s">
+      <c r="L1043" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1043" s="2" t="s">
@@ -21419,7 +21422,7 @@
       </c>
     </row>
     <row r="1044" ht="15.75" customHeight="1">
-      <c r="L1044" s="2" t="s">
+      <c r="L1044" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1044" s="2" t="s">
@@ -21436,7 +21439,7 @@
       </c>
     </row>
     <row r="1045" ht="15.75" customHeight="1">
-      <c r="L1045" s="2" t="s">
+      <c r="L1045" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1045" s="2" t="s">
@@ -21451,7 +21454,7 @@
       </c>
     </row>
     <row r="1046" ht="15.75" customHeight="1">
-      <c r="L1046" s="2" t="s">
+      <c r="L1046" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1046" s="2" t="s">
@@ -21468,7 +21471,7 @@
       </c>
     </row>
     <row r="1047" ht="15.75" customHeight="1">
-      <c r="L1047" s="2" t="s">
+      <c r="L1047" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1047" s="2" t="s">
@@ -21485,7 +21488,7 @@
       </c>
     </row>
     <row r="1048" ht="15.75" customHeight="1">
-      <c r="L1048" s="2" t="s">
+      <c r="L1048" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1048" s="2" t="s">
@@ -21500,7 +21503,7 @@
       </c>
     </row>
     <row r="1049" ht="15.75" customHeight="1">
-      <c r="L1049" s="2" t="s">
+      <c r="L1049" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1049" s="2" t="s">
@@ -21517,7 +21520,7 @@
       </c>
     </row>
     <row r="1050" ht="15.75" customHeight="1">
-      <c r="L1050" s="2" t="s">
+      <c r="L1050" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1050" s="2" t="s">
@@ -21532,7 +21535,7 @@
       </c>
     </row>
     <row r="1051" ht="15.75" customHeight="1">
-      <c r="L1051" s="2" t="s">
+      <c r="L1051" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1051" s="2" t="s">
@@ -21549,7 +21552,7 @@
       </c>
     </row>
     <row r="1052" ht="15.75" customHeight="1">
-      <c r="L1052" s="2" t="s">
+      <c r="L1052" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1052" s="2" t="s">
@@ -21564,7 +21567,7 @@
       </c>
     </row>
     <row r="1053" ht="15.75" customHeight="1">
-      <c r="L1053" s="2" t="s">
+      <c r="L1053" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1053" s="2" t="s">
@@ -21579,7 +21582,7 @@
       </c>
     </row>
     <row r="1054" ht="15.75" customHeight="1">
-      <c r="L1054" s="2" t="s">
+      <c r="L1054" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1054" s="2" t="s">
@@ -21596,7 +21599,7 @@
       </c>
     </row>
     <row r="1055" ht="15.75" customHeight="1">
-      <c r="L1055" s="2" t="s">
+      <c r="L1055" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1055" s="2" t="s">
@@ -21611,7 +21614,7 @@
       </c>
     </row>
     <row r="1056" ht="15.75" customHeight="1">
-      <c r="L1056" s="2" t="s">
+      <c r="L1056" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1056" s="2" t="s">
@@ -21628,7 +21631,7 @@
       </c>
     </row>
     <row r="1057" ht="15.75" customHeight="1">
-      <c r="L1057" s="2" t="s">
+      <c r="L1057" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1057" s="2" t="s">
@@ -21645,7 +21648,7 @@
       </c>
     </row>
     <row r="1058" ht="15.75" customHeight="1">
-      <c r="L1058" s="2" t="s">
+      <c r="L1058" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1058" s="2" t="s">
@@ -21662,7 +21665,7 @@
       </c>
     </row>
     <row r="1059" ht="15.75" customHeight="1">
-      <c r="L1059" s="2" t="s">
+      <c r="L1059" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1059" s="2" t="s">
@@ -21679,7 +21682,7 @@
       </c>
     </row>
     <row r="1060" ht="15.75" customHeight="1">
-      <c r="L1060" s="2" t="s">
+      <c r="L1060" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1060" s="2" t="s">
@@ -21696,7 +21699,7 @@
       </c>
     </row>
     <row r="1061" ht="15.75" customHeight="1">
-      <c r="L1061" s="2" t="s">
+      <c r="L1061" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1061" s="2" t="s">
@@ -21713,7 +21716,7 @@
       </c>
     </row>
     <row r="1062" ht="15.75" customHeight="1">
-      <c r="L1062" s="2" t="s">
+      <c r="L1062" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1062" s="2" t="s">
@@ -21730,7 +21733,7 @@
       </c>
     </row>
     <row r="1063" ht="15.75" customHeight="1">
-      <c r="L1063" s="2" t="s">
+      <c r="L1063" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1063" s="2" t="s">
@@ -21745,7 +21748,7 @@
       </c>
     </row>
     <row r="1064" ht="15.75" customHeight="1">
-      <c r="L1064" s="2" t="s">
+      <c r="L1064" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1064" s="2" t="s">
@@ -21762,7 +21765,7 @@
       </c>
     </row>
     <row r="1065" ht="15.75" customHeight="1">
-      <c r="L1065" s="2" t="s">
+      <c r="L1065" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1065" s="2" t="s">
@@ -21779,7 +21782,7 @@
       </c>
     </row>
     <row r="1066" ht="15.75" customHeight="1">
-      <c r="L1066" s="2" t="s">
+      <c r="L1066" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1066" s="2" t="s">
@@ -21796,7 +21799,7 @@
       </c>
     </row>
     <row r="1067" ht="15.75" customHeight="1">
-      <c r="L1067" s="2" t="s">
+      <c r="L1067" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1067" s="2" t="s">
@@ -21813,7 +21816,7 @@
       </c>
     </row>
     <row r="1068" ht="15.75" customHeight="1">
-      <c r="L1068" s="2" t="s">
+      <c r="L1068" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1068" s="2" t="s">
@@ -21830,7 +21833,7 @@
       </c>
     </row>
     <row r="1069" ht="15.75" customHeight="1">
-      <c r="L1069" s="2" t="s">
+      <c r="L1069" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1069" s="2" t="s">
@@ -21845,7 +21848,7 @@
       </c>
     </row>
     <row r="1070" ht="15.75" customHeight="1">
-      <c r="L1070" s="2" t="s">
+      <c r="L1070" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1070" s="2" t="s">
@@ -21862,7 +21865,7 @@
       </c>
     </row>
     <row r="1071" ht="15.75" customHeight="1">
-      <c r="L1071" s="2" t="s">
+      <c r="L1071" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1071" s="2" t="s">
@@ -21879,7 +21882,7 @@
       </c>
     </row>
     <row r="1072" ht="15.75" customHeight="1">
-      <c r="L1072" s="2" t="s">
+      <c r="L1072" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1072" s="2" t="s">
@@ -21894,7 +21897,7 @@
       </c>
     </row>
     <row r="1073" ht="15.75" customHeight="1">
-      <c r="L1073" s="2" t="s">
+      <c r="L1073" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1073" s="2" t="s">
@@ -21909,7 +21912,7 @@
       </c>
     </row>
     <row r="1074" ht="15.75" customHeight="1">
-      <c r="L1074" s="2" t="s">
+      <c r="L1074" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1074" s="2" t="s">
@@ -21926,7 +21929,7 @@
       </c>
     </row>
     <row r="1075" ht="15.75" customHeight="1">
-      <c r="L1075" s="2" t="s">
+      <c r="L1075" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1075" s="2" t="s">
@@ -21941,7 +21944,7 @@
       </c>
     </row>
     <row r="1076" ht="15.75" customHeight="1">
-      <c r="L1076" s="2" t="s">
+      <c r="L1076" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1076" s="2" t="s">
@@ -21958,7 +21961,7 @@
       </c>
     </row>
     <row r="1077" ht="15.75" customHeight="1">
-      <c r="L1077" s="2" t="s">
+      <c r="L1077" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1077" s="2" t="s">
@@ -21973,7 +21976,7 @@
       </c>
     </row>
     <row r="1078" ht="15.75" customHeight="1">
-      <c r="L1078" s="2" t="s">
+      <c r="L1078" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1078" s="2" t="s">
@@ -21988,7 +21991,7 @@
       </c>
     </row>
     <row r="1079" ht="15.75" customHeight="1">
-      <c r="L1079" s="2" t="s">
+      <c r="L1079" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1079" s="2" t="s">
@@ -22005,7 +22008,7 @@
       </c>
     </row>
     <row r="1080" ht="15.75" customHeight="1">
-      <c r="L1080" s="2" t="s">
+      <c r="L1080" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1080" s="2" t="s">
@@ -22022,7 +22025,7 @@
       </c>
     </row>
     <row r="1081" ht="15.75" customHeight="1">
-      <c r="L1081" s="2" t="s">
+      <c r="L1081" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1081" s="2" t="s">
@@ -22039,7 +22042,7 @@
       </c>
     </row>
     <row r="1082" ht="15.75" customHeight="1">
-      <c r="L1082" s="2" t="s">
+      <c r="L1082" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1082" s="2" t="s">
@@ -22056,7 +22059,7 @@
       </c>
     </row>
     <row r="1083" ht="15.75" customHeight="1">
-      <c r="L1083" s="2" t="s">
+      <c r="L1083" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1083" s="2" t="s">
@@ -22073,7 +22076,7 @@
       </c>
     </row>
     <row r="1084" ht="15.75" customHeight="1">
-      <c r="L1084" s="2" t="s">
+      <c r="L1084" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1084" s="2" t="s">
@@ -22090,7 +22093,7 @@
       </c>
     </row>
     <row r="1085" ht="15.75" customHeight="1">
-      <c r="L1085" s="2" t="s">
+      <c r="L1085" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1085" s="2" t="s">
@@ -22107,7 +22110,7 @@
       </c>
     </row>
     <row r="1086" ht="15.75" customHeight="1">
-      <c r="L1086" s="2" t="s">
+      <c r="L1086" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1086" s="2" t="s">
@@ -22124,7 +22127,7 @@
       </c>
     </row>
     <row r="1087" ht="15.75" customHeight="1">
-      <c r="L1087" s="2" t="s">
+      <c r="L1087" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1087" s="2" t="s">
@@ -22141,7 +22144,7 @@
       </c>
     </row>
     <row r="1088" ht="15.75" customHeight="1">
-      <c r="L1088" s="2" t="s">
+      <c r="L1088" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1088" s="2" t="s">
@@ -22158,7 +22161,7 @@
       </c>
     </row>
     <row r="1089" ht="15.75" customHeight="1">
-      <c r="L1089" s="2" t="s">
+      <c r="L1089" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1089" s="2" t="s">
@@ -22173,7 +22176,7 @@
       </c>
     </row>
     <row r="1090" ht="15.75" customHeight="1">
-      <c r="L1090" s="2" t="s">
+      <c r="L1090" s="3" t="s">
         <v>741</v>
       </c>
       <c r="M1090" s="2" t="s">
@@ -22188,7 +22191,7 @@
       </c>
     </row>
     <row r="1091" ht="15.75" customHeight="1">
-      <c r="L1091" s="2" t="s">
+      <c r="L1091" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1091" s="2" t="s">
@@ -22205,7 +22208,7 @@
       </c>
     </row>
     <row r="1092" ht="15.75" customHeight="1">
-      <c r="L1092" s="2" t="s">
+      <c r="L1092" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1092" s="2" t="s">
@@ -22222,7 +22225,7 @@
       </c>
     </row>
     <row r="1093" ht="15.75" customHeight="1">
-      <c r="L1093" s="2" t="s">
+      <c r="L1093" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1093" s="2" t="s">
@@ -22237,7 +22240,7 @@
       </c>
     </row>
     <row r="1094" ht="15.75" customHeight="1">
-      <c r="L1094" s="2" t="s">
+      <c r="L1094" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1094" s="2" t="s">
@@ -22252,7 +22255,7 @@
       </c>
     </row>
     <row r="1095" ht="15.75" customHeight="1">
-      <c r="L1095" s="2" t="s">
+      <c r="L1095" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1095" s="2" t="s">
@@ -22267,7 +22270,7 @@
       </c>
     </row>
     <row r="1096" ht="15.75" customHeight="1">
-      <c r="L1096" s="2" t="s">
+      <c r="L1096" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1096" s="2" t="s">
@@ -22282,7 +22285,7 @@
       </c>
     </row>
     <row r="1097" ht="15.75" customHeight="1">
-      <c r="L1097" s="2" t="s">
+      <c r="L1097" s="3" t="s">
         <v>747</v>
       </c>
       <c r="M1097" s="2" t="s">
@@ -22299,7 +22302,7 @@
       </c>
     </row>
     <row r="1098" ht="15.75" customHeight="1">
-      <c r="L1098" s="2" t="s">
+      <c r="L1098" s="3" t="s">
         <v>747</v>
       </c>
       <c r="M1098" s="2" t="s">
@@ -22312,7 +22315,7 @@
       </c>
     </row>
     <row r="1099" ht="15.75" customHeight="1">
-      <c r="L1099" s="2" t="s">
+      <c r="L1099" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1099" s="2" t="s">
@@ -22329,7 +22332,7 @@
       </c>
     </row>
     <row r="1100" ht="15.75" customHeight="1">
-      <c r="L1100" s="2" t="s">
+      <c r="L1100" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1100" s="2" t="s">
@@ -22346,7 +22349,7 @@
       </c>
     </row>
     <row r="1101" ht="15.75" customHeight="1">
-      <c r="L1101" s="2" t="s">
+      <c r="L1101" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1101" s="2" t="s">
@@ -22363,7 +22366,7 @@
       </c>
     </row>
     <row r="1102" ht="15.75" customHeight="1">
-      <c r="L1102" s="2" t="s">
+      <c r="L1102" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1102" s="2" t="s">
@@ -22380,7 +22383,7 @@
       </c>
     </row>
     <row r="1103" ht="15.75" customHeight="1">
-      <c r="L1103" s="2" t="s">
+      <c r="L1103" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1103" s="2" t="s">
@@ -22397,7 +22400,7 @@
       </c>
     </row>
     <row r="1104" ht="15.75" customHeight="1">
-      <c r="L1104" s="2" t="s">
+      <c r="L1104" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1104" s="2" t="s">
@@ -22414,7 +22417,7 @@
       </c>
     </row>
     <row r="1105" ht="15.75" customHeight="1">
-      <c r="L1105" s="2" t="s">
+      <c r="L1105" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1105" s="2" t="s">
@@ -22431,7 +22434,7 @@
       </c>
     </row>
     <row r="1106" ht="15.75" customHeight="1">
-      <c r="L1106" s="2" t="s">
+      <c r="L1106" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1106" s="2" t="s">
@@ -22448,7 +22451,7 @@
       </c>
     </row>
     <row r="1107" ht="15.75" customHeight="1">
-      <c r="L1107" s="2" t="s">
+      <c r="L1107" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1107" s="2" t="s">
@@ -22463,7 +22466,7 @@
       </c>
     </row>
     <row r="1108" ht="15.75" customHeight="1">
-      <c r="L1108" s="2" t="s">
+      <c r="L1108" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1108" s="2" t="s">
@@ -22480,7 +22483,7 @@
       </c>
     </row>
     <row r="1109" ht="15.75" customHeight="1">
-      <c r="L1109" s="2" t="s">
+      <c r="L1109" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1109" s="2" t="s">
@@ -22495,7 +22498,7 @@
       </c>
     </row>
     <row r="1110" ht="15.75" customHeight="1">
-      <c r="L1110" s="2" t="s">
+      <c r="L1110" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1110" s="2" t="s">
@@ -22510,7 +22513,7 @@
       </c>
     </row>
     <row r="1111" ht="15.75" customHeight="1">
-      <c r="L1111" s="2" t="s">
+      <c r="L1111" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1111" s="2" t="s">
@@ -22527,7 +22530,7 @@
       </c>
     </row>
     <row r="1112" ht="15.75" customHeight="1">
-      <c r="L1112" s="2" t="s">
+      <c r="L1112" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1112" s="2" t="s">
@@ -22544,7 +22547,7 @@
       </c>
     </row>
     <row r="1113" ht="15.75" customHeight="1">
-      <c r="L1113" s="2" t="s">
+      <c r="L1113" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1113" s="2" t="s">
@@ -22561,7 +22564,7 @@
       </c>
     </row>
     <row r="1114" ht="15.75" customHeight="1">
-      <c r="L1114" s="2" t="s">
+      <c r="L1114" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1114" s="2" t="s">
@@ -22578,7 +22581,7 @@
       </c>
     </row>
     <row r="1115" ht="15.75" customHeight="1">
-      <c r="L1115" s="2" t="s">
+      <c r="L1115" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1115" s="2" t="s">
@@ -22595,7 +22598,7 @@
       </c>
     </row>
     <row r="1116" ht="15.75" customHeight="1">
-      <c r="L1116" s="2" t="s">
+      <c r="L1116" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1116" s="2" t="s">
@@ -22612,7 +22615,7 @@
       </c>
     </row>
     <row r="1117" ht="15.75" customHeight="1">
-      <c r="L1117" s="2" t="s">
+      <c r="L1117" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1117" s="2" t="s">
@@ -22629,7 +22632,7 @@
       </c>
     </row>
     <row r="1118" ht="15.75" customHeight="1">
-      <c r="L1118" s="2" t="s">
+      <c r="L1118" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1118" s="2" t="s">
@@ -22646,7 +22649,7 @@
       </c>
     </row>
     <row r="1119" ht="15.75" customHeight="1">
-      <c r="L1119" s="2" t="s">
+      <c r="L1119" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1119" s="2" t="s">
@@ -22663,7 +22666,7 @@
       </c>
     </row>
     <row r="1120" ht="15.75" customHeight="1">
-      <c r="L1120" s="2" t="s">
+      <c r="L1120" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1120" s="2" t="s">
@@ -22680,7 +22683,7 @@
       </c>
     </row>
     <row r="1121" ht="15.75" customHeight="1">
-      <c r="L1121" s="2" t="s">
+      <c r="L1121" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1121" s="2" t="s">
@@ -22697,7 +22700,7 @@
       </c>
     </row>
     <row r="1122" ht="15.75" customHeight="1">
-      <c r="L1122" s="2" t="s">
+      <c r="L1122" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1122" s="2" t="s">
@@ -22714,7 +22717,7 @@
       </c>
     </row>
     <row r="1123" ht="15.75" customHeight="1">
-      <c r="L1123" s="2" t="s">
+      <c r="L1123" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1123" s="2" t="s">
@@ -22731,7 +22734,7 @@
       </c>
     </row>
     <row r="1124" ht="15.75" customHeight="1">
-      <c r="L1124" s="2" t="s">
+      <c r="L1124" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1124" s="2" t="s">
@@ -22746,7 +22749,7 @@
       </c>
     </row>
     <row r="1125" ht="15.75" customHeight="1">
-      <c r="L1125" s="2" t="s">
+      <c r="L1125" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1125" s="2" t="s">
@@ -22763,7 +22766,7 @@
       </c>
     </row>
     <row r="1126" ht="15.75" customHeight="1">
-      <c r="L1126" s="2" t="s">
+      <c r="L1126" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1126" s="2" t="s">
@@ -22780,7 +22783,7 @@
       </c>
     </row>
     <row r="1127" ht="15.75" customHeight="1">
-      <c r="L1127" s="2" t="s">
+      <c r="L1127" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1127" s="2" t="s">
@@ -22797,7 +22800,7 @@
       </c>
     </row>
     <row r="1128" ht="15.75" customHeight="1">
-      <c r="L1128" s="2" t="s">
+      <c r="L1128" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1128" s="2" t="s">
@@ -22814,7 +22817,7 @@
       </c>
     </row>
     <row r="1129" ht="15.75" customHeight="1">
-      <c r="L1129" s="2" t="s">
+      <c r="L1129" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1129" s="2" t="s">
@@ -22829,7 +22832,7 @@
       </c>
     </row>
     <row r="1130" ht="15.75" customHeight="1">
-      <c r="L1130" s="2" t="s">
+      <c r="L1130" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1130" s="2" t="s">
@@ -22844,7 +22847,7 @@
       </c>
     </row>
     <row r="1131" ht="15.75" customHeight="1">
-      <c r="L1131" s="2" t="s">
+      <c r="L1131" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1131" s="2" t="s">
@@ -22859,7 +22862,7 @@
       </c>
     </row>
     <row r="1132" ht="15.75" customHeight="1">
-      <c r="L1132" s="2" t="s">
+      <c r="L1132" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1132" s="2" t="s">
@@ -22876,7 +22879,7 @@
       </c>
     </row>
     <row r="1133" ht="15.75" customHeight="1">
-      <c r="L1133" s="2" t="s">
+      <c r="L1133" s="3" t="s">
         <v>747</v>
       </c>
       <c r="M1133" s="2" t="s">
@@ -22893,7 +22896,7 @@
       </c>
     </row>
     <row r="1134" ht="15.75" customHeight="1">
-      <c r="L1134" s="2" t="s">
+      <c r="L1134" s="3" t="s">
         <v>747</v>
       </c>
       <c r="M1134" s="2" t="s">
@@ -22910,7 +22913,7 @@
       </c>
     </row>
     <row r="1135" ht="15.75" customHeight="1">
-      <c r="L1135" s="2" t="s">
+      <c r="L1135" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1135" s="2" t="s">
@@ -22927,7 +22930,7 @@
       </c>
     </row>
     <row r="1136" ht="15.75" customHeight="1">
-      <c r="L1136" s="2" t="s">
+      <c r="L1136" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1136" s="2" t="s">
@@ -22944,7 +22947,7 @@
       </c>
     </row>
     <row r="1137" ht="15.75" customHeight="1">
-      <c r="L1137" s="2" t="s">
+      <c r="L1137" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1137" s="2" t="s">
@@ -22961,7 +22964,7 @@
       </c>
     </row>
     <row r="1138" ht="15.75" customHeight="1">
-      <c r="L1138" s="2" t="s">
+      <c r="L1138" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1138" s="2" t="s">
@@ -22978,7 +22981,7 @@
       </c>
     </row>
     <row r="1139" ht="15.75" customHeight="1">
-      <c r="L1139" s="2" t="s">
+      <c r="L1139" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1139" s="2" t="s">
@@ -22995,7 +22998,7 @@
       </c>
     </row>
     <row r="1140" ht="15.75" customHeight="1">
-      <c r="L1140" s="2" t="s">
+      <c r="L1140" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1140" s="2" t="s">
@@ -23012,7 +23015,7 @@
       </c>
     </row>
     <row r="1141" ht="15.75" customHeight="1">
-      <c r="L1141" s="2" t="s">
+      <c r="L1141" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1141" s="2" t="s">
@@ -23029,7 +23032,7 @@
       </c>
     </row>
     <row r="1142" ht="15.75" customHeight="1">
-      <c r="L1142" s="2" t="s">
+      <c r="L1142" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1142" s="2" t="s">
@@ -23046,7 +23049,7 @@
       </c>
     </row>
     <row r="1143" ht="15.75" customHeight="1">
-      <c r="L1143" s="2" t="s">
+      <c r="L1143" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1143" s="2" t="s">
@@ -23063,7 +23066,7 @@
       </c>
     </row>
     <row r="1144" ht="15.75" customHeight="1">
-      <c r="L1144" s="2" t="s">
+      <c r="L1144" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1144" s="2" t="s">
@@ -23080,7 +23083,7 @@
       </c>
     </row>
     <row r="1145" ht="15.75" customHeight="1">
-      <c r="L1145" s="2" t="s">
+      <c r="L1145" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1145" s="2" t="s">
@@ -23097,7 +23100,7 @@
       </c>
     </row>
     <row r="1146" ht="15.75" customHeight="1">
-      <c r="L1146" s="2" t="s">
+      <c r="L1146" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1146" s="2" t="s">
@@ -23114,7 +23117,7 @@
       </c>
     </row>
     <row r="1147" ht="15.75" customHeight="1">
-      <c r="L1147" s="2" t="s">
+      <c r="L1147" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1147" s="2" t="s">
@@ -23131,7 +23134,7 @@
       </c>
     </row>
     <row r="1148" ht="15.75" customHeight="1">
-      <c r="L1148" s="2" t="s">
+      <c r="L1148" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1148" s="2" t="s">
@@ -23148,7 +23151,7 @@
       </c>
     </row>
     <row r="1149" ht="15.75" customHeight="1">
-      <c r="L1149" s="2" t="s">
+      <c r="L1149" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1149" s="2" t="s">
@@ -23165,7 +23168,7 @@
       </c>
     </row>
     <row r="1150" ht="15.75" customHeight="1">
-      <c r="L1150" s="2" t="s">
+      <c r="L1150" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1150" s="2" t="s">
@@ -23182,7 +23185,7 @@
       </c>
     </row>
     <row r="1151" ht="15.75" customHeight="1">
-      <c r="L1151" s="2" t="s">
+      <c r="L1151" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1151" s="2" t="s">
@@ -23199,7 +23202,7 @@
       </c>
     </row>
     <row r="1152" ht="15.75" customHeight="1">
-      <c r="L1152" s="2" t="s">
+      <c r="L1152" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1152" s="2" t="s">
@@ -23216,7 +23219,7 @@
       </c>
     </row>
     <row r="1153" ht="15.75" customHeight="1">
-      <c r="L1153" s="2" t="s">
+      <c r="L1153" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1153" s="2" t="s">
@@ -23233,7 +23236,7 @@
       </c>
     </row>
     <row r="1154" ht="15.75" customHeight="1">
-      <c r="L1154" s="2" t="s">
+      <c r="L1154" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1154" s="2" t="s">
@@ -23250,7 +23253,7 @@
       </c>
     </row>
     <row r="1155" ht="15.75" customHeight="1">
-      <c r="L1155" s="2" t="s">
+      <c r="L1155" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1155" s="2" t="s">
@@ -23267,7 +23270,7 @@
       </c>
     </row>
     <row r="1156" ht="15.75" customHeight="1">
-      <c r="L1156" s="2" t="s">
+      <c r="L1156" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1156" s="2" t="s">
@@ -23284,7 +23287,7 @@
       </c>
     </row>
     <row r="1157" ht="15.75" customHeight="1">
-      <c r="L1157" s="2" t="s">
+      <c r="L1157" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1157" s="2" t="s">
@@ -23301,7 +23304,7 @@
       </c>
     </row>
     <row r="1158" ht="15.75" customHeight="1">
-      <c r="L1158" s="2" t="s">
+      <c r="L1158" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1158" s="2" t="s">
@@ -23318,7 +23321,7 @@
       </c>
     </row>
     <row r="1159" ht="15.75" customHeight="1">
-      <c r="L1159" s="2" t="s">
+      <c r="L1159" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1159" s="2" t="s">
@@ -23335,7 +23338,7 @@
       </c>
     </row>
     <row r="1160" ht="15.75" customHeight="1">
-      <c r="L1160" s="2" t="s">
+      <c r="L1160" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1160" s="2" t="s">
@@ -23352,7 +23355,7 @@
       </c>
     </row>
     <row r="1161" ht="15.75" customHeight="1">
-      <c r="L1161" s="2" t="s">
+      <c r="L1161" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1161" s="2" t="s">
@@ -23369,7 +23372,7 @@
       </c>
     </row>
     <row r="1162" ht="15.75" customHeight="1">
-      <c r="L1162" s="2" t="s">
+      <c r="L1162" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1162" s="2" t="s">
@@ -23384,7 +23387,7 @@
       </c>
     </row>
     <row r="1163" ht="15.75" customHeight="1">
-      <c r="L1163" s="2" t="s">
+      <c r="L1163" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1163" s="2" t="s">
@@ -23401,7 +23404,7 @@
       </c>
     </row>
     <row r="1164" ht="15.75" customHeight="1">
-      <c r="L1164" s="2" t="s">
+      <c r="L1164" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1164" s="2" t="s">
@@ -23418,7 +23421,7 @@
       </c>
     </row>
     <row r="1165" ht="15.75" customHeight="1">
-      <c r="L1165" s="2" t="s">
+      <c r="L1165" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1165" s="2" t="s">
@@ -23435,7 +23438,7 @@
       </c>
     </row>
     <row r="1166" ht="15.75" customHeight="1">
-      <c r="L1166" s="2" t="s">
+      <c r="L1166" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1166" s="2" t="s">
@@ -23452,7 +23455,7 @@
       </c>
     </row>
     <row r="1167" ht="15.75" customHeight="1">
-      <c r="L1167" s="2" t="s">
+      <c r="L1167" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1167" s="2" t="s">
@@ -23469,7 +23472,7 @@
       </c>
     </row>
     <row r="1168" ht="15.75" customHeight="1">
-      <c r="L1168" s="2" t="s">
+      <c r="L1168" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1168" s="2" t="s">
@@ -23486,7 +23489,7 @@
       </c>
     </row>
     <row r="1169" ht="15.75" customHeight="1">
-      <c r="L1169" s="2" t="s">
+      <c r="L1169" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1169" s="2" t="s">
@@ -23503,7 +23506,7 @@
       </c>
     </row>
     <row r="1170" ht="15.75" customHeight="1">
-      <c r="L1170" s="2" t="s">
+      <c r="L1170" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1170" s="2" t="s">
@@ -23520,7 +23523,7 @@
       </c>
     </row>
     <row r="1171" ht="15.75" customHeight="1">
-      <c r="L1171" s="2" t="s">
+      <c r="L1171" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1171" s="2" t="s">
@@ -23537,7 +23540,7 @@
       </c>
     </row>
     <row r="1172" ht="15.75" customHeight="1">
-      <c r="L1172" s="2" t="s">
+      <c r="L1172" s="3" t="s">
         <v>741</v>
       </c>
       <c r="M1172" s="2" t="s">
@@ -23554,7 +23557,7 @@
       </c>
     </row>
     <row r="1173" ht="15.75" customHeight="1">
-      <c r="L1173" s="2" t="s">
+      <c r="L1173" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1173" s="2" t="s">
@@ -23571,7 +23574,7 @@
       </c>
     </row>
     <row r="1174" ht="15.75" customHeight="1">
-      <c r="L1174" s="2" t="s">
+      <c r="L1174" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1174" s="2" t="s">
@@ -23588,7 +23591,7 @@
       </c>
     </row>
     <row r="1175" ht="15.75" customHeight="1">
-      <c r="L1175" s="2" t="s">
+      <c r="L1175" s="3" t="s">
         <v>747</v>
       </c>
       <c r="M1175" s="2" t="s">
@@ -23605,7 +23608,7 @@
       </c>
     </row>
     <row r="1176" ht="15.75" customHeight="1">
-      <c r="L1176" s="2" t="s">
+      <c r="L1176" s="3" t="s">
         <v>793</v>
       </c>
       <c r="M1176" s="2" t="s">
@@ -23622,7 +23625,7 @@
       </c>
     </row>
     <row r="1177" ht="15.75" customHeight="1">
-      <c r="L1177" s="2" t="s">
+      <c r="L1177" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1177" s="2" t="s">
@@ -23639,7 +23642,7 @@
       </c>
     </row>
     <row r="1178" ht="15.75" customHeight="1">
-      <c r="L1178" s="2" t="s">
+      <c r="L1178" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1178" s="2" t="s">
@@ -23656,7 +23659,7 @@
       </c>
     </row>
     <row r="1179" ht="15.75" customHeight="1">
-      <c r="L1179" s="2" t="s">
+      <c r="L1179" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1179" s="2" t="s">
@@ -23673,7 +23676,7 @@
       </c>
     </row>
     <row r="1180" ht="15.75" customHeight="1">
-      <c r="L1180" s="2" t="s">
+      <c r="L1180" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1180" s="2" t="s">
@@ -23690,7 +23693,7 @@
       </c>
     </row>
     <row r="1181" ht="15.75" customHeight="1">
-      <c r="L1181" s="2" t="s">
+      <c r="L1181" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1181" s="2" t="s">
@@ -23707,7 +23710,7 @@
       </c>
     </row>
     <row r="1182" ht="15.75" customHeight="1">
-      <c r="L1182" s="2" t="s">
+      <c r="L1182" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1182" s="2" t="s">
@@ -23724,7 +23727,7 @@
       </c>
     </row>
     <row r="1183" ht="15.75" customHeight="1">
-      <c r="L1183" s="2" t="s">
+      <c r="L1183" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1183" s="2" t="s">
@@ -23741,7 +23744,7 @@
       </c>
     </row>
     <row r="1184" ht="15.75" customHeight="1">
-      <c r="L1184" s="2" t="s">
+      <c r="L1184" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1184" s="2" t="s">
@@ -23758,7 +23761,7 @@
       </c>
     </row>
     <row r="1185" ht="15.75" customHeight="1">
-      <c r="L1185" s="2" t="s">
+      <c r="L1185" s="3" t="s">
         <v>747</v>
       </c>
       <c r="M1185" s="2" t="s">
@@ -23775,7 +23778,7 @@
       </c>
     </row>
     <row r="1186" ht="15.75" customHeight="1">
-      <c r="L1186" s="2" t="s">
+      <c r="L1186" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1186" s="2" t="s">
@@ -23792,7 +23795,7 @@
       </c>
     </row>
     <row r="1187" ht="15.75" customHeight="1">
-      <c r="L1187" s="2" t="s">
+      <c r="L1187" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1187" s="2" t="s">
@@ -23809,7 +23812,7 @@
       </c>
     </row>
     <row r="1188" ht="15.75" customHeight="1">
-      <c r="L1188" s="2" t="s">
+      <c r="L1188" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1188" s="2" t="s">
@@ -23826,7 +23829,7 @@
       </c>
     </row>
     <row r="1189" ht="15.75" customHeight="1">
-      <c r="L1189" s="2" t="s">
+      <c r="L1189" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1189" s="2" t="s">
@@ -23843,7 +23846,7 @@
       </c>
     </row>
     <row r="1190" ht="15.75" customHeight="1">
-      <c r="L1190" s="2" t="s">
+      <c r="L1190" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1190" s="2" t="s">
@@ -23860,7 +23863,7 @@
       </c>
     </row>
     <row r="1191" ht="15.75" customHeight="1">
-      <c r="L1191" s="2" t="s">
+      <c r="L1191" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1191" s="2" t="s">
@@ -23877,7 +23880,7 @@
       </c>
     </row>
     <row r="1192" ht="15.75" customHeight="1">
-      <c r="L1192" s="2" t="s">
+      <c r="L1192" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1192" s="2" t="s">
@@ -23894,7 +23897,7 @@
       </c>
     </row>
     <row r="1193" ht="15.75" customHeight="1">
-      <c r="L1193" s="2" t="s">
+      <c r="L1193" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1193" s="2" t="s">
@@ -23911,7 +23914,7 @@
       </c>
     </row>
     <row r="1194" ht="15.75" customHeight="1">
-      <c r="L1194" s="2" t="s">
+      <c r="L1194" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1194" s="2" t="s">
@@ -23928,7 +23931,7 @@
       </c>
     </row>
     <row r="1195" ht="15.75" customHeight="1">
-      <c r="L1195" s="2" t="s">
+      <c r="L1195" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1195" s="2" t="s">
@@ -23945,7 +23948,7 @@
       </c>
     </row>
     <row r="1196" ht="15.75" customHeight="1">
-      <c r="L1196" s="2" t="s">
+      <c r="L1196" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1196" s="2" t="s">
@@ -23962,7 +23965,7 @@
       </c>
     </row>
     <row r="1197" ht="15.75" customHeight="1">
-      <c r="L1197" s="2" t="s">
+      <c r="L1197" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1197" s="2" t="s">
@@ -23979,7 +23982,7 @@
       </c>
     </row>
     <row r="1198" ht="15.75" customHeight="1">
-      <c r="L1198" s="2" t="s">
+      <c r="L1198" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1198" s="2" t="s">
@@ -23996,7 +23999,7 @@
       </c>
     </row>
     <row r="1199" ht="15.75" customHeight="1">
-      <c r="L1199" s="2" t="s">
+      <c r="L1199" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1199" s="2" t="s">
@@ -24011,7 +24014,7 @@
       </c>
     </row>
     <row r="1200" ht="15.75" customHeight="1">
-      <c r="L1200" s="2" t="s">
+      <c r="L1200" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1200" s="2" t="s">
@@ -24028,7 +24031,7 @@
       </c>
     </row>
     <row r="1201" ht="15.75" customHeight="1">
-      <c r="L1201" s="2" t="s">
+      <c r="L1201" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1201" s="2" t="s">
@@ -24045,7 +24048,7 @@
       </c>
     </row>
     <row r="1202" ht="15.75" customHeight="1">
-      <c r="L1202" s="2" t="s">
+      <c r="L1202" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1202" s="2" t="s">
@@ -24062,7 +24065,7 @@
       </c>
     </row>
     <row r="1203" ht="15.75" customHeight="1">
-      <c r="L1203" s="2" t="s">
+      <c r="L1203" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1203" s="2" t="s">
@@ -24079,7 +24082,7 @@
       </c>
     </row>
     <row r="1204" ht="15.75" customHeight="1">
-      <c r="L1204" s="2" t="s">
+      <c r="L1204" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1204" s="2" t="s">
@@ -24096,7 +24099,7 @@
       </c>
     </row>
     <row r="1205" ht="15.75" customHeight="1">
-      <c r="L1205" s="2" t="s">
+      <c r="L1205" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1205" s="2" t="s">
@@ -24113,7 +24116,7 @@
       </c>
     </row>
     <row r="1206" ht="15.75" customHeight="1">
-      <c r="L1206" s="2" t="s">
+      <c r="L1206" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1206" s="2" t="s">
@@ -24130,7 +24133,7 @@
       </c>
     </row>
     <row r="1207" ht="15.75" customHeight="1">
-      <c r="L1207" s="2" t="s">
+      <c r="L1207" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1207" s="2" t="s">
@@ -24145,7 +24148,7 @@
       </c>
     </row>
     <row r="1208" ht="15.75" customHeight="1">
-      <c r="L1208" s="2" t="s">
+      <c r="L1208" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1208" s="2" t="s">
@@ -24160,7 +24163,7 @@
       </c>
     </row>
     <row r="1209" ht="15.75" customHeight="1">
-      <c r="L1209" s="2" t="s">
+      <c r="L1209" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1209" s="2" t="s">
@@ -24175,7 +24178,7 @@
       </c>
     </row>
     <row r="1210" ht="15.75" customHeight="1">
-      <c r="L1210" s="2" t="s">
+      <c r="L1210" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1210" s="2" t="s">
@@ -24190,7 +24193,7 @@
       </c>
     </row>
     <row r="1211" ht="15.75" customHeight="1">
-      <c r="L1211" s="2" t="s">
+      <c r="L1211" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1211" s="2" t="s">
@@ -24207,7 +24210,7 @@
       </c>
     </row>
     <row r="1212" ht="15.75" customHeight="1">
-      <c r="L1212" s="2" t="s">
+      <c r="L1212" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1212" s="2" t="s">
@@ -24224,7 +24227,7 @@
       </c>
     </row>
     <row r="1213" ht="15.75" customHeight="1">
-      <c r="L1213" s="2" t="s">
+      <c r="L1213" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1213" s="2" t="s">
@@ -24241,7 +24244,7 @@
       </c>
     </row>
     <row r="1214" ht="15.75" customHeight="1">
-      <c r="L1214" s="2" t="s">
+      <c r="L1214" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1214" s="2" t="s">
@@ -24258,7 +24261,7 @@
       </c>
     </row>
     <row r="1215" ht="15.75" customHeight="1">
-      <c r="L1215" s="2" t="s">
+      <c r="L1215" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1215" s="2" t="s">
@@ -24275,7 +24278,7 @@
       </c>
     </row>
     <row r="1216" ht="15.75" customHeight="1">
-      <c r="L1216" s="2" t="s">
+      <c r="L1216" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1216" s="2" t="s">
@@ -24292,7 +24295,7 @@
       </c>
     </row>
     <row r="1217" ht="15.75" customHeight="1">
-      <c r="L1217" s="2" t="s">
+      <c r="L1217" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1217" s="2" t="s">
@@ -24309,7 +24312,7 @@
       </c>
     </row>
     <row r="1218" ht="15.75" customHeight="1">
-      <c r="L1218" s="2" t="s">
+      <c r="L1218" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1218" s="2" t="s">
@@ -24322,7 +24325,7 @@
       </c>
     </row>
     <row r="1219" ht="15.75" customHeight="1">
-      <c r="L1219" s="2" t="s">
+      <c r="L1219" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1219" s="2" t="s">
@@ -24335,7 +24338,7 @@
       </c>
     </row>
     <row r="1220" ht="15.75" customHeight="1">
-      <c r="L1220" s="2" t="s">
+      <c r="L1220" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1220" s="2" t="s">
@@ -24352,7 +24355,7 @@
       </c>
     </row>
     <row r="1221" ht="15.75" customHeight="1">
-      <c r="L1221" s="2" t="s">
+      <c r="L1221" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1221" s="2" t="s">
@@ -24369,7 +24372,7 @@
       </c>
     </row>
     <row r="1222" ht="15.75" customHeight="1">
-      <c r="L1222" s="2" t="s">
+      <c r="L1222" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1222" s="2" t="s">
@@ -24386,7 +24389,7 @@
       </c>
     </row>
     <row r="1223" ht="15.75" customHeight="1">
-      <c r="L1223" s="2" t="s">
+      <c r="L1223" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1223" s="2" t="s">
@@ -24403,7 +24406,7 @@
       </c>
     </row>
     <row r="1224" ht="15.75" customHeight="1">
-      <c r="L1224" s="2" t="s">
+      <c r="L1224" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1224" s="2" t="s">
@@ -24420,7 +24423,7 @@
       </c>
     </row>
     <row r="1225" ht="15.75" customHeight="1">
-      <c r="L1225" s="2" t="s">
+      <c r="L1225" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1225" s="2" t="s">
@@ -24437,7 +24440,7 @@
       </c>
     </row>
     <row r="1226" ht="15.75" customHeight="1">
-      <c r="L1226" s="2" t="s">
+      <c r="L1226" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1226" s="2" t="s">
@@ -24454,7 +24457,7 @@
       </c>
     </row>
     <row r="1227" ht="15.75" customHeight="1">
-      <c r="L1227" s="2" t="s">
+      <c r="L1227" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1227" s="2" t="s">
@@ -24471,7 +24474,7 @@
       </c>
     </row>
     <row r="1228" ht="15.75" customHeight="1">
-      <c r="L1228" s="2" t="s">
+      <c r="L1228" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1228" s="2" t="s">
@@ -24488,7 +24491,7 @@
       </c>
     </row>
     <row r="1229" ht="15.75" customHeight="1">
-      <c r="L1229" s="2" t="s">
+      <c r="L1229" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1229" s="2" t="s">
@@ -24505,7 +24508,7 @@
       </c>
     </row>
     <row r="1230" ht="15.75" customHeight="1">
-      <c r="L1230" s="2" t="s">
+      <c r="L1230" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1230" s="2" t="s">
@@ -24522,7 +24525,7 @@
       </c>
     </row>
     <row r="1231" ht="15.75" customHeight="1">
-      <c r="L1231" s="2" t="s">
+      <c r="L1231" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1231" s="2" t="s">
@@ -24539,7 +24542,7 @@
       </c>
     </row>
     <row r="1232" ht="15.75" customHeight="1">
-      <c r="L1232" s="2" t="s">
+      <c r="L1232" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1232" s="2" t="s">
@@ -24556,7 +24559,7 @@
       </c>
     </row>
     <row r="1233" ht="15.75" customHeight="1">
-      <c r="L1233" s="2" t="s">
+      <c r="L1233" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1233" s="2" t="s">
@@ -24571,7 +24574,7 @@
       </c>
     </row>
     <row r="1234" ht="15.75" customHeight="1">
-      <c r="L1234" s="2" t="s">
+      <c r="L1234" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1234" s="2" t="s">
@@ -24588,7 +24591,7 @@
       </c>
     </row>
     <row r="1235" ht="15.75" customHeight="1">
-      <c r="L1235" s="2" t="s">
+      <c r="L1235" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1235" s="2" t="s">
@@ -24605,7 +24608,7 @@
       </c>
     </row>
     <row r="1236" ht="15.75" customHeight="1">
-      <c r="L1236" s="2" t="s">
+      <c r="L1236" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1236" s="2" t="s">
@@ -24622,7 +24625,7 @@
       </c>
     </row>
     <row r="1237" ht="15.75" customHeight="1">
-      <c r="L1237" s="2" t="s">
+      <c r="L1237" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1237" s="2" t="s">
@@ -24639,7 +24642,7 @@
       </c>
     </row>
     <row r="1238" ht="15.75" customHeight="1">
-      <c r="L1238" s="2" t="s">
+      <c r="L1238" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1238" s="2" t="s">
@@ -24656,7 +24659,7 @@
       </c>
     </row>
     <row r="1239" ht="15.75" customHeight="1">
-      <c r="L1239" s="2" t="s">
+      <c r="L1239" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1239" s="2" t="s">
@@ -24673,7 +24676,7 @@
       </c>
     </row>
     <row r="1240" ht="15.75" customHeight="1">
-      <c r="L1240" s="2" t="s">
+      <c r="L1240" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1240" s="2" t="s">
@@ -24688,7 +24691,7 @@
       </c>
     </row>
     <row r="1241" ht="15.75" customHeight="1">
-      <c r="L1241" s="2" t="s">
+      <c r="L1241" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1241" s="2" t="s">
@@ -24705,7 +24708,7 @@
       </c>
     </row>
     <row r="1242" ht="15.75" customHeight="1">
-      <c r="L1242" s="2" t="s">
+      <c r="L1242" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1242" s="2" t="s">
@@ -24722,7 +24725,7 @@
       </c>
     </row>
     <row r="1243" ht="15.75" customHeight="1">
-      <c r="L1243" s="2" t="s">
+      <c r="L1243" s="3" t="s">
         <v>747</v>
       </c>
       <c r="M1243" s="2" t="s">
@@ -24739,7 +24742,7 @@
       </c>
     </row>
     <row r="1244" ht="15.75" customHeight="1">
-      <c r="L1244" s="2" t="s">
+      <c r="L1244" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1244" s="2" t="s">
@@ -24752,7 +24755,7 @@
       </c>
     </row>
     <row r="1245" ht="15.75" customHeight="1">
-      <c r="L1245" s="2" t="s">
+      <c r="L1245" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1245" s="2" t="s">
@@ -24769,7 +24772,7 @@
       </c>
     </row>
     <row r="1246" ht="15.75" customHeight="1">
-      <c r="L1246" s="2" t="s">
+      <c r="L1246" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1246" s="2" t="s">
@@ -24786,7 +24789,7 @@
       </c>
     </row>
     <row r="1247" ht="15.75" customHeight="1">
-      <c r="L1247" s="2" t="s">
+      <c r="L1247" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1247" s="2" t="s">
@@ -24803,7 +24806,7 @@
       </c>
     </row>
     <row r="1248" ht="15.75" customHeight="1">
-      <c r="L1248" s="2" t="s">
+      <c r="L1248" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1248" s="2" t="s">
@@ -24820,7 +24823,7 @@
       </c>
     </row>
     <row r="1249" ht="15.75" customHeight="1">
-      <c r="L1249" s="2" t="s">
+      <c r="L1249" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1249" s="2" t="s">
@@ -24837,7 +24840,7 @@
       </c>
     </row>
     <row r="1250" ht="15.75" customHeight="1">
-      <c r="L1250" s="2" t="s">
+      <c r="L1250" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1250" s="2" t="s">
@@ -24854,7 +24857,7 @@
       </c>
     </row>
     <row r="1251" ht="15.75" customHeight="1">
-      <c r="L1251" s="2" t="s">
+      <c r="L1251" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1251" s="2" t="s">
@@ -24871,7 +24874,7 @@
       </c>
     </row>
     <row r="1252" ht="15.75" customHeight="1">
-      <c r="L1252" s="2" t="s">
+      <c r="L1252" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1252" s="2" t="s">
@@ -24888,7 +24891,7 @@
       </c>
     </row>
     <row r="1253" ht="15.75" customHeight="1">
-      <c r="L1253" s="2" t="s">
+      <c r="L1253" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1253" s="2" t="s">
@@ -24905,7 +24908,7 @@
       </c>
     </row>
     <row r="1254" ht="15.75" customHeight="1">
-      <c r="L1254" s="2" t="s">
+      <c r="L1254" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1254" s="2" t="s">
@@ -24922,7 +24925,7 @@
       </c>
     </row>
     <row r="1255" ht="15.75" customHeight="1">
-      <c r="L1255" s="2" t="s">
+      <c r="L1255" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1255" s="2" t="s">
@@ -24939,7 +24942,7 @@
       </c>
     </row>
     <row r="1256" ht="15.75" customHeight="1">
-      <c r="L1256" s="2" t="s">
+      <c r="L1256" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1256" s="2" t="s">
@@ -24956,7 +24959,7 @@
       </c>
     </row>
     <row r="1257" ht="15.75" customHeight="1">
-      <c r="L1257" s="2" t="s">
+      <c r="L1257" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1257" s="2" t="s">
@@ -24973,7 +24976,7 @@
       </c>
     </row>
     <row r="1258" ht="15.75" customHeight="1">
-      <c r="L1258" s="2" t="s">
+      <c r="L1258" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1258" s="2" t="s">
@@ -24990,7 +24993,7 @@
       </c>
     </row>
     <row r="1259" ht="15.75" customHeight="1">
-      <c r="L1259" s="2" t="s">
+      <c r="L1259" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1259" s="2" t="s">
@@ -25007,7 +25010,7 @@
       </c>
     </row>
     <row r="1260" ht="15.75" customHeight="1">
-      <c r="L1260" s="2" t="s">
+      <c r="L1260" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1260" s="2" t="s">
@@ -25024,7 +25027,7 @@
       </c>
     </row>
     <row r="1261" ht="15.75" customHeight="1">
-      <c r="L1261" s="2" t="s">
+      <c r="L1261" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1261" s="2" t="s">
@@ -25041,7 +25044,7 @@
       </c>
     </row>
     <row r="1262" ht="15.75" customHeight="1">
-      <c r="L1262" s="2" t="s">
+      <c r="L1262" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1262" s="2" t="s">
@@ -25058,7 +25061,7 @@
       </c>
     </row>
     <row r="1263" ht="15.75" customHeight="1">
-      <c r="L1263" s="2" t="s">
+      <c r="L1263" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1263" s="2" t="s">
@@ -25075,7 +25078,7 @@
       </c>
     </row>
     <row r="1264" ht="15.75" customHeight="1">
-      <c r="L1264" s="2" t="s">
+      <c r="L1264" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1264" s="2" t="s">
@@ -25092,7 +25095,7 @@
       </c>
     </row>
     <row r="1265" ht="15.75" customHeight="1">
-      <c r="L1265" s="2" t="s">
+      <c r="L1265" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1265" s="2" t="s">
@@ -25109,7 +25112,7 @@
       </c>
     </row>
     <row r="1266" ht="15.75" customHeight="1">
-      <c r="L1266" s="2" t="s">
+      <c r="L1266" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1266" s="2" t="s">
@@ -25124,7 +25127,7 @@
       </c>
     </row>
     <row r="1267" ht="15.75" customHeight="1">
-      <c r="L1267" s="2" t="s">
+      <c r="L1267" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1267" s="2" t="s">
@@ -25141,7 +25144,7 @@
       </c>
     </row>
     <row r="1268" ht="15.75" customHeight="1">
-      <c r="L1268" s="2" t="s">
+      <c r="L1268" s="3" t="s">
         <v>747</v>
       </c>
       <c r="M1268" s="2" t="s">
@@ -25158,7 +25161,7 @@
       </c>
     </row>
     <row r="1269" ht="15.75" customHeight="1">
-      <c r="L1269" s="2" t="s">
+      <c r="L1269" s="3" t="s">
         <v>747</v>
       </c>
       <c r="M1269" s="2" t="s">
@@ -25175,7 +25178,7 @@
       </c>
     </row>
     <row r="1270" ht="15.75" customHeight="1">
-      <c r="L1270" s="2" t="s">
+      <c r="L1270" s="3" t="s">
         <v>747</v>
       </c>
       <c r="M1270" s="2" t="s">
@@ -25192,7 +25195,7 @@
       </c>
     </row>
     <row r="1271" ht="15.75" customHeight="1">
-      <c r="L1271" s="2" t="s">
+      <c r="L1271" s="3" t="s">
         <v>747</v>
       </c>
       <c r="M1271" s="2" t="s">
@@ -25209,7 +25212,7 @@
       </c>
     </row>
     <row r="1272" ht="15.75" customHeight="1">
-      <c r="L1272" s="2" t="s">
+      <c r="L1272" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1272" s="2" t="s">
@@ -25226,7 +25229,7 @@
       </c>
     </row>
     <row r="1273" ht="15.75" customHeight="1">
-      <c r="L1273" s="2" t="s">
+      <c r="L1273" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1273" s="2" t="s">
@@ -25241,7 +25244,7 @@
       </c>
     </row>
     <row r="1274" ht="15.75" customHeight="1">
-      <c r="L1274" s="2" t="s">
+      <c r="L1274" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1274" s="2"/>
@@ -25252,7 +25255,7 @@
       </c>
     </row>
     <row r="1275" ht="15.75" customHeight="1">
-      <c r="L1275" s="2" t="s">
+      <c r="L1275" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1275" s="2" t="s">
@@ -25267,7 +25270,7 @@
       </c>
     </row>
     <row r="1276" ht="15.75" customHeight="1">
-      <c r="L1276" s="2" t="s">
+      <c r="L1276" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1276" s="2" t="s">
@@ -25284,7 +25287,7 @@
       </c>
     </row>
     <row r="1277" ht="15.75" customHeight="1">
-      <c r="L1277" s="2" t="s">
+      <c r="L1277" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1277" s="2" t="s">
@@ -25299,7 +25302,7 @@
       </c>
     </row>
     <row r="1278" ht="15.75" customHeight="1">
-      <c r="L1278" s="2" t="s">
+      <c r="L1278" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1278" s="2"/>
@@ -25310,7 +25313,7 @@
       </c>
     </row>
     <row r="1279" ht="15.75" customHeight="1">
-      <c r="L1279" s="2" t="s">
+      <c r="L1279" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1279" s="2"/>
@@ -25321,7 +25324,7 @@
       </c>
     </row>
     <row r="1280" ht="15.75" customHeight="1">
-      <c r="L1280" s="2" t="s">
+      <c r="L1280" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1280" s="2" t="s">
@@ -25336,7 +25339,7 @@
       </c>
     </row>
     <row r="1281" ht="15.75" customHeight="1">
-      <c r="L1281" s="2" t="s">
+      <c r="L1281" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1281" s="2" t="s">
@@ -25349,7 +25352,7 @@
       </c>
     </row>
     <row r="1282" ht="15.75" customHeight="1">
-      <c r="L1282" s="2" t="s">
+      <c r="L1282" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1282" s="2" t="s">
@@ -25364,7 +25367,7 @@
       </c>
     </row>
     <row r="1283" ht="15.75" customHeight="1">
-      <c r="L1283" s="2" t="s">
+      <c r="L1283" s="3" t="s">
         <v>741</v>
       </c>
       <c r="M1283" s="2" t="s">
@@ -25381,7 +25384,7 @@
       </c>
     </row>
     <row r="1284" ht="15.75" customHeight="1">
-      <c r="L1284" s="2" t="s">
+      <c r="L1284" s="3" t="s">
         <v>741</v>
       </c>
       <c r="M1284" s="2" t="s">
@@ -25398,7 +25401,7 @@
       </c>
     </row>
     <row r="1285" ht="15.75" customHeight="1">
-      <c r="L1285" s="2" t="s">
+      <c r="L1285" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1285" s="2" t="s">
@@ -25415,7 +25418,7 @@
       </c>
     </row>
     <row r="1286" ht="15.75" customHeight="1">
-      <c r="L1286" s="2" t="s">
+      <c r="L1286" s="3" t="s">
         <v>741</v>
       </c>
       <c r="M1286" s="2" t="s">
@@ -25432,7 +25435,7 @@
       </c>
     </row>
     <row r="1287" ht="15.75" customHeight="1">
-      <c r="L1287" s="2" t="s">
+      <c r="L1287" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1287" s="2" t="s">
@@ -25449,7 +25452,7 @@
       </c>
     </row>
     <row r="1288" ht="15.75" customHeight="1">
-      <c r="L1288" s="2" t="s">
+      <c r="L1288" s="3" t="s">
         <v>747</v>
       </c>
       <c r="M1288" s="2" t="s">
@@ -25466,7 +25469,7 @@
       </c>
     </row>
     <row r="1289" ht="15.75" customHeight="1">
-      <c r="L1289" s="2" t="s">
+      <c r="L1289" s="3" t="s">
         <v>747</v>
       </c>
       <c r="M1289" s="2" t="s">
@@ -25483,7 +25486,7 @@
       </c>
     </row>
     <row r="1290" ht="15.75" customHeight="1">
-      <c r="L1290" s="2" t="s">
+      <c r="L1290" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1290" s="2" t="s">
@@ -25500,7 +25503,7 @@
       </c>
     </row>
     <row r="1291" ht="15.75" customHeight="1">
-      <c r="L1291" s="2" t="s">
+      <c r="L1291" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1291" s="2" t="s">
@@ -25517,7 +25520,7 @@
       </c>
     </row>
     <row r="1292" ht="15.75" customHeight="1">
-      <c r="L1292" s="2" t="s">
+      <c r="L1292" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1292" s="2" t="s">
@@ -25534,7 +25537,7 @@
       </c>
     </row>
     <row r="1293" ht="15.75" customHeight="1">
-      <c r="L1293" s="2" t="s">
+      <c r="L1293" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1293" s="2" t="s">
@@ -25551,7 +25554,7 @@
       </c>
     </row>
     <row r="1294" ht="15.75" customHeight="1">
-      <c r="L1294" s="2" t="s">
+      <c r="L1294" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1294" s="2" t="s">
@@ -25566,7 +25569,7 @@
       </c>
     </row>
     <row r="1295" ht="15.75" customHeight="1">
-      <c r="L1295" s="2" t="s">
+      <c r="L1295" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1295" s="2" t="s">
@@ -25581,7 +25584,7 @@
       </c>
     </row>
     <row r="1296" ht="15.75" customHeight="1">
-      <c r="L1296" s="2" t="s">
+      <c r="L1296" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1296" s="2" t="s">
@@ -25596,7 +25599,7 @@
       </c>
     </row>
     <row r="1297" ht="15.75" customHeight="1">
-      <c r="L1297" s="2" t="s">
+      <c r="L1297" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1297" s="2" t="s">
@@ -25613,7 +25616,7 @@
       </c>
     </row>
     <row r="1298" ht="15.75" customHeight="1">
-      <c r="L1298" s="2" t="s">
+      <c r="L1298" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1298" s="2" t="s">
@@ -25630,7 +25633,7 @@
       </c>
     </row>
     <row r="1299" ht="15.75" customHeight="1">
-      <c r="L1299" s="2" t="s">
+      <c r="L1299" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1299" s="2" t="s">
@@ -25647,7 +25650,7 @@
       </c>
     </row>
     <row r="1300" ht="15.75" customHeight="1">
-      <c r="L1300" s="2" t="s">
+      <c r="L1300" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1300" s="2" t="s">
@@ -25664,7 +25667,7 @@
       </c>
     </row>
     <row r="1301" ht="15.75" customHeight="1">
-      <c r="L1301" s="2" t="s">
+      <c r="L1301" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1301" s="2" t="s">
@@ -25679,7 +25682,7 @@
       </c>
     </row>
     <row r="1302" ht="15.75" customHeight="1">
-      <c r="L1302" s="2" t="s">
+      <c r="L1302" s="3" t="s">
         <v>747</v>
       </c>
       <c r="M1302" s="2" t="s">
@@ -25696,7 +25699,7 @@
       </c>
     </row>
     <row r="1303" ht="15.75" customHeight="1">
-      <c r="L1303" s="2" t="s">
+      <c r="L1303" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1303" s="2" t="s">
@@ -25713,7 +25716,7 @@
       </c>
     </row>
     <row r="1304" ht="15.75" customHeight="1">
-      <c r="L1304" s="2" t="s">
+      <c r="L1304" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1304" s="2" t="s">
@@ -25730,7 +25733,7 @@
       </c>
     </row>
     <row r="1305" ht="15.75" customHeight="1">
-      <c r="L1305" s="2" t="s">
+      <c r="L1305" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1305" s="2" t="s">
@@ -25747,7 +25750,7 @@
       </c>
     </row>
     <row r="1306" ht="15.75" customHeight="1">
-      <c r="L1306" s="2" t="s">
+      <c r="L1306" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1306" s="2" t="s">
@@ -25764,7 +25767,7 @@
       </c>
     </row>
     <row r="1307" ht="15.75" customHeight="1">
-      <c r="L1307" s="2" t="s">
+      <c r="L1307" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1307" s="2" t="s">
@@ -25781,7 +25784,7 @@
       </c>
     </row>
     <row r="1308" ht="15.75" customHeight="1">
-      <c r="L1308" s="2" t="s">
+      <c r="L1308" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1308" s="2" t="s">
@@ -25798,7 +25801,7 @@
       </c>
     </row>
     <row r="1309" ht="15.75" customHeight="1">
-      <c r="L1309" s="2" t="s">
+      <c r="L1309" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1309" s="2" t="s">
@@ -25815,7 +25818,7 @@
       </c>
     </row>
     <row r="1310" ht="15.75" customHeight="1">
-      <c r="L1310" s="2" t="s">
+      <c r="L1310" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1310" s="2" t="s">
@@ -25832,7 +25835,7 @@
       </c>
     </row>
     <row r="1311" ht="15.75" customHeight="1">
-      <c r="L1311" s="2" t="s">
+      <c r="L1311" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1311" s="2" t="s">
@@ -25849,7 +25852,7 @@
       </c>
     </row>
     <row r="1312" ht="15.75" customHeight="1">
-      <c r="L1312" s="2" t="s">
+      <c r="L1312" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1312" s="2" t="s">
@@ -25866,7 +25869,7 @@
       </c>
     </row>
     <row r="1313" ht="15.75" customHeight="1">
-      <c r="L1313" s="2" t="s">
+      <c r="L1313" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1313" s="2" t="s">
@@ -25883,7 +25886,7 @@
       </c>
     </row>
     <row r="1314" ht="15.75" customHeight="1">
-      <c r="L1314" s="2" t="s">
+      <c r="L1314" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1314" s="2" t="s">
@@ -25900,7 +25903,7 @@
       </c>
     </row>
     <row r="1315" ht="15.75" customHeight="1">
-      <c r="L1315" s="2" t="s">
+      <c r="L1315" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1315" s="2" t="s">
@@ -25917,7 +25920,7 @@
       </c>
     </row>
     <row r="1316" ht="15.75" customHeight="1">
-      <c r="L1316" s="2" t="s">
+      <c r="L1316" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1316" s="2" t="s">
@@ -25934,7 +25937,7 @@
       </c>
     </row>
     <row r="1317" ht="15.75" customHeight="1">
-      <c r="L1317" s="2" t="s">
+      <c r="L1317" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1317" s="2" t="s">
@@ -25951,7 +25954,7 @@
       </c>
     </row>
     <row r="1318" ht="15.75" customHeight="1">
-      <c r="L1318" s="2" t="s">
+      <c r="L1318" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1318" s="2" t="s">
@@ -25968,7 +25971,7 @@
       </c>
     </row>
     <row r="1319" ht="15.75" customHeight="1">
-      <c r="L1319" s="2" t="s">
+      <c r="L1319" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1319" s="2" t="s">
@@ -25985,7 +25988,7 @@
       </c>
     </row>
     <row r="1320" ht="15.75" customHeight="1">
-      <c r="L1320" s="2" t="s">
+      <c r="L1320" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1320" s="2" t="s">
@@ -26002,7 +26005,7 @@
       </c>
     </row>
     <row r="1321" ht="15.75" customHeight="1">
-      <c r="L1321" s="2" t="s">
+      <c r="L1321" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1321" s="2" t="s">
@@ -26019,7 +26022,7 @@
       </c>
     </row>
     <row r="1322" ht="15.75" customHeight="1">
-      <c r="L1322" s="2" t="s">
+      <c r="L1322" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1322" s="2" t="s">
@@ -26036,7 +26039,7 @@
       </c>
     </row>
     <row r="1323" ht="15.75" customHeight="1">
-      <c r="L1323" s="2" t="s">
+      <c r="L1323" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1323" s="2" t="s">
@@ -26053,7 +26056,7 @@
       </c>
     </row>
     <row r="1324" ht="15.75" customHeight="1">
-      <c r="L1324" s="2" t="s">
+      <c r="L1324" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1324" s="2" t="s">
@@ -26068,7 +26071,7 @@
       </c>
     </row>
     <row r="1325" ht="15.75" customHeight="1">
-      <c r="L1325" s="2" t="s">
+      <c r="L1325" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1325" s="2" t="s">
@@ -26083,7 +26086,7 @@
       </c>
     </row>
     <row r="1326" ht="15.75" customHeight="1">
-      <c r="L1326" s="2" t="s">
+      <c r="L1326" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1326" s="2" t="s">
@@ -26100,7 +26103,7 @@
       </c>
     </row>
     <row r="1327" ht="15.75" customHeight="1">
-      <c r="L1327" s="2" t="s">
+      <c r="L1327" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1327" s="2" t="s">
@@ -26115,7 +26118,7 @@
       </c>
     </row>
     <row r="1328" ht="15.75" customHeight="1">
-      <c r="L1328" s="2" t="s">
+      <c r="L1328" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1328" s="2" t="s">
@@ -26132,7 +26135,7 @@
       </c>
     </row>
     <row r="1329" ht="15.75" customHeight="1">
-      <c r="L1329" s="2" t="s">
+      <c r="L1329" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1329" s="2" t="s">
@@ -26147,7 +26150,7 @@
       </c>
     </row>
     <row r="1330" ht="15.75" customHeight="1">
-      <c r="L1330" s="2" t="s">
+      <c r="L1330" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1330" s="2" t="s">
@@ -26162,7 +26165,7 @@
       </c>
     </row>
     <row r="1331" ht="15.75" customHeight="1">
-      <c r="L1331" s="2" t="s">
+      <c r="L1331" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1331" s="2" t="s">
@@ -26177,7 +26180,7 @@
       </c>
     </row>
     <row r="1332" ht="15.75" customHeight="1">
-      <c r="L1332" s="2" t="s">
+      <c r="L1332" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1332" s="2" t="s">
@@ -26192,7 +26195,7 @@
       </c>
     </row>
     <row r="1333" ht="15.75" customHeight="1">
-      <c r="L1333" s="2" t="s">
+      <c r="L1333" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1333" s="2" t="s">
@@ -26209,7 +26212,7 @@
       </c>
     </row>
     <row r="1334" ht="15.75" customHeight="1">
-      <c r="L1334" s="2" t="s">
+      <c r="L1334" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1334" s="2" t="s">
@@ -26226,7 +26229,7 @@
       </c>
     </row>
     <row r="1335" ht="15.75" customHeight="1">
-      <c r="L1335" s="2" t="s">
+      <c r="L1335" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1335" s="2" t="s">
@@ -26243,7 +26246,7 @@
       </c>
     </row>
     <row r="1336" ht="15.75" customHeight="1">
-      <c r="L1336" s="2" t="s">
+      <c r="L1336" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1336" s="2" t="s">
@@ -26260,7 +26263,7 @@
       </c>
     </row>
     <row r="1337" ht="15.75" customHeight="1">
-      <c r="L1337" s="2" t="s">
+      <c r="L1337" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1337" s="2" t="s">
@@ -26277,7 +26280,7 @@
       </c>
     </row>
     <row r="1338" ht="15.75" customHeight="1">
-      <c r="L1338" s="2" t="s">
+      <c r="L1338" s="3" t="s">
         <v>679</v>
       </c>
       <c r="M1338" s="2" t="s">
@@ -26294,7 +26297,7 @@
       </c>
     </row>
     <row r="1339" ht="15.75" customHeight="1">
-      <c r="L1339" s="2" t="s">
+      <c r="L1339" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1339" s="2" t="s">
@@ -26311,7 +26314,7 @@
       </c>
     </row>
     <row r="1340" ht="15.75" customHeight="1">
-      <c r="L1340" s="2" t="s">
+      <c r="L1340" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1340" s="2" t="s">
@@ -26328,7 +26331,7 @@
       </c>
     </row>
     <row r="1341" ht="15.75" customHeight="1">
-      <c r="L1341" s="2" t="s">
+      <c r="L1341" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1341" s="2" t="s">
@@ -26345,7 +26348,7 @@
       </c>
     </row>
     <row r="1342" ht="15.75" customHeight="1">
-      <c r="L1342" s="2" t="s">
+      <c r="L1342" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1342" s="2" t="s">
@@ -26362,7 +26365,7 @@
       </c>
     </row>
     <row r="1343" ht="15.75" customHeight="1">
-      <c r="L1343" s="2" t="s">
+      <c r="L1343" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1343" s="2" t="s">
@@ -26379,7 +26382,7 @@
       </c>
     </row>
     <row r="1344" ht="15.75" customHeight="1">
-      <c r="L1344" s="2" t="s">
+      <c r="L1344" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1344" s="2" t="s">
@@ -26396,7 +26399,7 @@
       </c>
     </row>
     <row r="1345" ht="15.75" customHeight="1">
-      <c r="L1345" s="2" t="s">
+      <c r="L1345" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1345" s="2" t="s">
@@ -26413,7 +26416,7 @@
       </c>
     </row>
     <row r="1346" ht="15.75" customHeight="1">
-      <c r="L1346" s="2" t="s">
+      <c r="L1346" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1346" s="2" t="s">
@@ -26430,7 +26433,7 @@
       </c>
     </row>
     <row r="1347" ht="15.75" customHeight="1">
-      <c r="L1347" s="2" t="s">
+      <c r="L1347" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1347" s="2" t="s">
@@ -26447,7 +26450,7 @@
       </c>
     </row>
     <row r="1348" ht="15.75" customHeight="1">
-      <c r="L1348" s="2" t="s">
+      <c r="L1348" s="3" t="s">
         <v>741</v>
       </c>
       <c r="M1348" s="2" t="s">
@@ -26464,7 +26467,7 @@
       </c>
     </row>
     <row r="1349" ht="15.75" customHeight="1">
-      <c r="L1349" s="2" t="s">
+      <c r="L1349" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1349" s="2" t="s">
@@ -26479,7 +26482,7 @@
       </c>
     </row>
     <row r="1350" ht="15.75" customHeight="1">
-      <c r="L1350" s="2" t="s">
+      <c r="L1350" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1350" s="2" t="s">
@@ -26494,7 +26497,7 @@
       </c>
     </row>
     <row r="1351" ht="15.75" customHeight="1">
-      <c r="L1351" s="2" t="s">
+      <c r="L1351" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1351" s="2" t="s">
@@ -26511,7 +26514,7 @@
       </c>
     </row>
     <row r="1352" ht="15.75" customHeight="1">
-      <c r="L1352" s="2" t="s">
+      <c r="L1352" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1352" s="2" t="s">
@@ -26528,7 +26531,7 @@
       </c>
     </row>
     <row r="1353" ht="15.75" customHeight="1">
-      <c r="L1353" s="2" t="s">
+      <c r="L1353" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1353" s="2" t="s">
@@ -26545,7 +26548,7 @@
       </c>
     </row>
     <row r="1354" ht="15.75" customHeight="1">
-      <c r="L1354" s="2" t="s">
+      <c r="L1354" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1354" s="2" t="s">
@@ -26562,7 +26565,7 @@
       </c>
     </row>
     <row r="1355" ht="15.75" customHeight="1">
-      <c r="L1355" s="2" t="s">
+      <c r="L1355" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1355" s="2" t="s">
@@ -26579,7 +26582,7 @@
       </c>
     </row>
     <row r="1356" ht="15.75" customHeight="1">
-      <c r="L1356" s="2" t="s">
+      <c r="L1356" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1356" s="2" t="s">
@@ -26596,7 +26599,7 @@
       </c>
     </row>
     <row r="1357" ht="15.75" customHeight="1">
-      <c r="L1357" s="2" t="s">
+      <c r="L1357" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1357" s="2" t="s">
@@ -26613,7 +26616,7 @@
       </c>
     </row>
     <row r="1358" ht="15.75" customHeight="1">
-      <c r="L1358" s="2" t="s">
+      <c r="L1358" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1358" s="2" t="s">
@@ -26630,7 +26633,7 @@
       </c>
     </row>
     <row r="1359" ht="15.75" customHeight="1">
-      <c r="L1359" s="2" t="s">
+      <c r="L1359" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1359" s="2" t="s">
@@ -26647,7 +26650,7 @@
       </c>
     </row>
     <row r="1360" ht="15.75" customHeight="1">
-      <c r="L1360" s="2" t="s">
+      <c r="L1360" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1360" s="2" t="s">
@@ -26664,7 +26667,7 @@
       </c>
     </row>
     <row r="1361" ht="15.75" customHeight="1">
-      <c r="L1361" s="2" t="s">
+      <c r="L1361" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1361" s="2" t="s">
@@ -26681,7 +26684,7 @@
       </c>
     </row>
     <row r="1362" ht="15.75" customHeight="1">
-      <c r="L1362" s="2" t="s">
+      <c r="L1362" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1362" s="2" t="s">
@@ -26698,7 +26701,7 @@
       </c>
     </row>
     <row r="1363" ht="15.75" customHeight="1">
-      <c r="L1363" s="2" t="s">
+      <c r="L1363" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1363" s="2" t="s">
@@ -26715,7 +26718,7 @@
       </c>
     </row>
     <row r="1364" ht="15.75" customHeight="1">
-      <c r="L1364" s="2" t="s">
+      <c r="L1364" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1364" s="2" t="s">
@@ -26732,7 +26735,7 @@
       </c>
     </row>
     <row r="1365" ht="15.75" customHeight="1">
-      <c r="L1365" s="2" t="s">
+      <c r="L1365" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1365" s="2" t="s">
@@ -26749,7 +26752,7 @@
       </c>
     </row>
     <row r="1366" ht="15.75" customHeight="1">
-      <c r="L1366" s="2" t="s">
+      <c r="L1366" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1366" s="2" t="s">
@@ -26766,7 +26769,7 @@
       </c>
     </row>
     <row r="1367" ht="15.75" customHeight="1">
-      <c r="L1367" s="2" t="s">
+      <c r="L1367" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1367" s="2" t="s">
@@ -26783,7 +26786,7 @@
       </c>
     </row>
     <row r="1368" ht="15.75" customHeight="1">
-      <c r="L1368" s="2" t="s">
+      <c r="L1368" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1368" s="2" t="s">
@@ -26800,7 +26803,7 @@
       </c>
     </row>
     <row r="1369" ht="15.75" customHeight="1">
-      <c r="L1369" s="2" t="s">
+      <c r="L1369" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1369" s="2" t="s">
@@ -26817,7 +26820,7 @@
       </c>
     </row>
     <row r="1370" ht="15.75" customHeight="1">
-      <c r="L1370" s="2" t="s">
+      <c r="L1370" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1370" s="2" t="s">
@@ -26834,7 +26837,7 @@
       </c>
     </row>
     <row r="1371" ht="15.75" customHeight="1">
-      <c r="L1371" s="2" t="s">
+      <c r="L1371" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1371" s="2" t="s">
@@ -26851,7 +26854,7 @@
       </c>
     </row>
     <row r="1372" ht="15.75" customHeight="1">
-      <c r="L1372" s="2" t="s">
+      <c r="L1372" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1372" s="2" t="s">
@@ -26868,7 +26871,7 @@
       </c>
     </row>
     <row r="1373" ht="15.75" customHeight="1">
-      <c r="L1373" s="2" t="s">
+      <c r="L1373" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1373" s="2" t="s">
@@ -26885,7 +26888,7 @@
       </c>
     </row>
     <row r="1374" ht="15.75" customHeight="1">
-      <c r="L1374" s="2" t="s">
+      <c r="L1374" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1374" s="2" t="s">
@@ -26900,7 +26903,7 @@
       </c>
     </row>
     <row r="1375" ht="15.75" customHeight="1">
-      <c r="L1375" s="2" t="s">
+      <c r="L1375" s="3" t="s">
         <v>793</v>
       </c>
       <c r="M1375" s="2" t="s">
@@ -26917,7 +26920,7 @@
       </c>
     </row>
     <row r="1376" ht="15.75" customHeight="1">
-      <c r="L1376" s="2" t="s">
+      <c r="L1376" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1376" s="2" t="s">
@@ -26934,7 +26937,7 @@
       </c>
     </row>
     <row r="1377" ht="15.75" customHeight="1">
-      <c r="L1377" s="2" t="s">
+      <c r="L1377" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1377" s="2" t="s">
@@ -26951,7 +26954,7 @@
       </c>
     </row>
     <row r="1378" ht="15.75" customHeight="1">
-      <c r="L1378" s="2" t="s">
+      <c r="L1378" s="3" t="s">
         <v>672</v>
       </c>
       <c r="M1378" s="2" t="s">

</xml_diff>